<commit_message>
Document email-mock behavior changes
</commit_message>
<xml_diff>
--- a/docs/test-plans/e2e_ui_test_matrix.xlsx
+++ b/docs/test-plans/e2e_ui_test_matrix.xlsx
@@ -57,14 +57,14 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="44" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="52" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1936,6 +1936,110 @@
       <c r="J36" t="inlineStr">
         <is>
           <t>Includes desktop site, mobile site menu, and admin sidebar navigation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>E36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Captured email API</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Mock email captures exact provider payload and preview routes return it</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Captured mock email exposes provider fields and the list/detail/raw HTML endpoints return the same payload for assertions and preview.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>apps/api-booking/test/dev-emails-preview.test.ts</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Assert against `from`, `replyTo`, `subject`, `text`, and `html` directly; do not use a fake preview abstraction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>E37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Dev email preview UI</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Browser preview renders captured HTML and real CTA links</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>`dev-emails.html` loads the captured email HTML in an iframe and exposes the real CTA hrefs for inspection.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Technical, S05, S07</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>apps/site/e2e/dev-emails-preview.spec.ts</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Spec added; deploy latest fixes before live verify</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Use `EMAIL_MODE=mock` and `ANTIBOT_MODE=mock`; rerun against a deployed target after shipping the latest worker/site changes.</t>
         </is>
       </c>
     </row>
@@ -1946,11 +2050,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="46" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1983,17 +2087,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>apps/site/e2e/navigation.smoke.spec.ts</t>
+          <t>apps/api-booking/test/dev-emails-preview.test.ts</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Desktop/mobile nav smoke plus admin sidebar runtime cleanliness</t>
+          <t>Captured email payload contract plus list/detail/raw HTML preview routes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- navigation.smoke.spec.ts</t>
+          <t>npm test -- dev-emails-preview.test.ts</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2003,24 +2107,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Best first smoke after frontend shell changes.</t>
+          <t>Smallest backend contract test for the new email-capture behavior.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>apps/site/e2e/booking-flows.spec.ts</t>
+          <t>apps/api-booking/test/booking-domain-model.test.ts</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Core free/pay-now/event happy paths</t>
+          <t>Booking orchestration with captured email assertions in real domain flows</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- booking-flows.spec.ts</t>
+          <t>npm test -- booking-domain-model.test.ts</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2030,24 +2134,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Desktop core-flow suite.</t>
+          <t>Includes regression assertions on captured email text/html content.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>apps/site/e2e/remaining-public.spec.ts</t>
+          <t>apps/site/e2e/navigation.smoke.spec.ts</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Remaining desktop public-state coverage</t>
+          <t>Desktop/mobile nav smoke plus admin sidebar runtime cleanliness</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- remaining-public.spec.ts</t>
+          <t>npm run test:e2e -- navigation.smoke.spec.ts</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2057,24 +2161,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Contains pay-later scenario that still needs refactor.</t>
+          <t>Best first smoke after frontend shell changes.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>apps/site/e2e/remaining-public.mobile.spec.ts</t>
+          <t>apps/site/e2e/booking-flows.spec.ts</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Remaining public-state mobile mirrors</t>
+          <t>Core free/pay-now/event happy paths</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- remaining-public.mobile.spec.ts</t>
+          <t>npm run test:e2e -- booking-flows.spec.ts</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2084,51 +2188,51 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mobile mirror wrapper over shared cases.</t>
+          <t>Desktop core-flow suite.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>apps/site/e2e/manage-admin.spec.ts</t>
+          <t>apps/site/e2e/dev-emails-preview.spec.ts</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Manage-link reschedule flows and one admin edit path</t>
+          <t>Browser preview of captured email HTML and real CTA links</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- manage-admin.spec.ts</t>
+          <t>npm run test:e2e -- dev-emails-preview.spec.ts</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Ready; verify after deploy</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Mixes self-service and admin behaviors.</t>
+          <t>Requires a target with the new `/api/__dev/emails` behavior deployed.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>apps/site/e2e/admin-remaining.spec.ts</t>
+          <t>apps/site/e2e/remaining-public.spec.ts</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Broader admin coverage for links, events, contact, content edits</t>
+          <t>Remaining desktop public-state coverage</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- admin-remaining.spec.ts</t>
+          <t>npm run test:e2e -- remaining-public.spec.ts</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2138,24 +2242,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Includes auth-required scenario currently fixme.</t>
+          <t>Contains pay-later scenario that still needs refactor.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>apps/site/e2e/contention.spec.ts</t>
+          <t>apps/site/e2e/remaining-public.mobile.spec.ts</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Two-user slot contention and stale-slot recovery</t>
+          <t>Remaining public-state mobile mirrors</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- contention.spec.ts</t>
+          <t>npm run test:e2e -- remaining-public.mobile.spec.ts</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2165,24 +2269,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Important booking-integrity regression suite.</t>
+          <t>Mobile mirror wrapper over shared cases.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>apps/site/e2e/mobile-regression.spec.ts</t>
+          <t>apps/site/e2e/manage-admin.spec.ts</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mobile mirrors of critical public flows</t>
+          <t>Manage-link reschedule flows and one admin edit path</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- mobile-regression.spec.ts --project mobile</t>
+          <t>npm run test:e2e -- manage-admin.spec.ts</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2192,24 +2296,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Main mobile path coverage.</t>
+          <t>Mixes self-service and admin behaviors.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>apps/site/e2e/turnstile-ui.spec.ts</t>
+          <t>apps/site/e2e/admin-remaining.spec.ts</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Turnstile booking/contact integration with mocked widget</t>
+          <t>Broader admin coverage for links, events, contact, content edits</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>npm run test:e2e -- turnstile-ui.spec.ts</t>
+          <t>npm run test:e2e -- admin-remaining.spec.ts</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2219,32 +2323,113 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>No external Turnstile dependency; fully mocked.</t>
+          <t>Includes auth-required scenario currently fixme.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>apps/site/e2e/contention.spec.ts</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Two-user slot contention and stale-slot recovery</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>npm run test:e2e -- contention.spec.ts</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Important booking-integrity regression suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>apps/site/e2e/mobile-regression.spec.ts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mobile mirrors of critical public flows</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>npm run test:e2e -- mobile-regression.spec.ts --project mobile</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Main mobile path coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>apps/site/e2e/turnstile-ui.spec.ts</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Turnstile booking/contact integration with mocked widget</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>npm run test:e2e -- turnstile-ui.spec.ts</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No external Turnstile dependency; fully mocked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>apps/site/e2e/pay-later-refactor.spec.ts</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Manual arrangement, settlement, expiry, and continue-payment behavior</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>npm run test:e2e -- pay-later-refactor.spec.ts</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Needs refactor</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Contains stale assumptions from before the 2026-03-15 pay-later refinement.</t>
         </is>
@@ -2259,7 +2444,7 @@
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2343,7 +2528,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mock inbox or live delivery environment.</t>
+          <t>Use `mock` for captured-email preview and payload inspection; `resend` disables `/api/__dev/emails*` as a preview source.</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2562,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mock or Turnstile-backed execution.</t>
+          <t>Use `mock` for deterministic email-preview booking setup.</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2586,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Intro offer URL</t>
+          <t>Latest fixes deployed?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2411,14 +2596,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Known-good public intro booking entry point.</t>
+          <t>Set this before running the browser email-preview spec against a live target.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Paid session offer URL</t>
+          <t>Intro offer URL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2428,14 +2613,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Known-good public paid session entry point.</t>
+          <t>Known-good public intro booking entry point.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Free event URL</t>
+          <t>Paid session offer URL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2445,14 +2630,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Known-good public free evening entry point.</t>
+          <t>Known-good public paid session entry point.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Paid event URL</t>
+          <t>Free event URL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2462,14 +2647,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Known-good public paid evening entry point.</t>
+          <t>Known-good public free evening entry point.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Valid manage link</t>
+          <t>Paid event URL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2479,14 +2664,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Reusable manage-link fixture for smoke checks.</t>
+          <t>Known-good public paid evening entry point.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Expired manage link</t>
+          <t>Valid manage link</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2496,14 +2681,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fixture for explicit invalid/expired handling.</t>
+          <t>Reusable manage-link fixture for smoke checks.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Valid confirmation link</t>
+          <t>Expired manage link</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2513,14 +2698,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fixture for confirmation-path checks.</t>
+          <t>Fixture for explicit invalid/expired handling.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Expired confirmation link</t>
+          <t>Valid confirmation link</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2530,14 +2715,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fixture for expiry-path checks.</t>
+          <t>Fixture for confirmation-path checks.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Valid late-access link</t>
+          <t>Expired confirmation link</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2547,14 +2732,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fixture for late-access booking checks.</t>
+          <t>Fixture for expiry-path checks.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rotated or expired late-access link</t>
+          <t>Valid late-access link</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2564,22 +2749,39 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fixture for revoked-token checks.</t>
+          <t>Fixture for late-access booking checks.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Rotated or expired late-access link</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fixture for revoked-token checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Notes location</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Bug tracker, spreadsheet, or text log used during execution.</t>
         </is>

</xml_diff>

<commit_message>
Add latest run status to plan
</commit_message>
<xml_diff>
--- a/docs/test-plans/e2e_ui_test_matrix.xlsx
+++ b/docs/test-plans/e2e_ui_test_matrix.xlsx
@@ -54,6 +54,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:L38"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -65,6 +66,8 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="58" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -118,6 +121,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>Latest Run Status</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t>Latest Run Comments</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -170,6 +183,16 @@
           <t>Runtime-clean coverage.</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -222,6 +245,16 @@
           <t>Structural public-state coverage.</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -274,6 +307,16 @@
           <t>Environment-dependent; returns early if no sold-out event exists.</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -326,6 +369,16 @@
           <t>Admin-mutates timing temporarily inside the test.</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -378,6 +431,16 @@
           <t>Covers unavailable-evening reminder path.</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -430,6 +493,16 @@
           <t>UI-validation coverage.</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -482,6 +555,16 @@
           <t>Also covered with Turnstile enabled in E33.</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -534,6 +617,16 @@
           <t>Strong end-to-end coverage across booking, confirm, manage, cancel.</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -586,6 +679,16 @@
           <t>Currently uses mock checkout path in E2E.</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -638,6 +741,16 @@
           <t>Current automation still contains stale submit-time pay-later assumptions and must be updated to the 2026-03-15 contract.</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -690,6 +803,16 @@
           <t>Uses currently available free public event.</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -742,6 +865,16 @@
           <t>Skipped automatically if no paid public event exists.</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -794,6 +927,16 @@
           <t>Admin rotates/creates late-access first.</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -846,6 +989,16 @@
           <t>Confirms no false positive payment completion.</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -898,6 +1051,16 @@
           <t>Allows expected 410 diagnostic noise.</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -950,6 +1113,16 @@
           <t>Allows expected 400 diagnostic noise.</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1002,6 +1175,16 @@
           <t>Core self-service reschedule path.</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1054,6 +1237,16 @@
           <t>Multi-booking setup; protects tricky slot-availability UX.</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1106,6 +1299,16 @@
           <t>Basic booking mutation coverage.</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1158,6 +1361,16 @@
           <t>Depends on created confirmed intro booking.</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1210,6 +1423,16 @@
           <t>Clipboard-dependent browser test.</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1262,6 +1485,16 @@
           <t>Popup-based coverage.</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1314,6 +1547,16 @@
           <t>Protects link revocation semantics.</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1366,6 +1609,16 @@
           <t>Covers public-to-admin message pipeline.</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1418,6 +1671,16 @@
           <t>Content-management coverage.</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1470,6 +1733,16 @@
           <t>Uses tiny in-memory JPEG payload.</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1522,6 +1795,16 @@
           <t>Skips if no editable event exists.</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1574,6 +1857,16 @@
           <t>Current pre-prod environment keeps admin auth disabled, so the test is intentionally not meaningful until auth is restored.</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1626,6 +1919,16 @@
           <t>High-value multi-user regression.</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1678,6 +1981,16 @@
           <t>Connects recovery UX with support fallback.</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1730,6 +2043,16 @@
           <t>Core anti-double-booking regression.</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1782,6 +2105,16 @@
           <t>Form-level antibot behavior with mocked config and fake widget.</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1834,6 +2167,16 @@
           <t>Covers anti-bot integration on contact flow.</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1886,6 +2229,16 @@
           <t>Technical UI guardrail rather than direct product requirement.</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1938,6 +2291,16 @@
           <t>Includes desktop site, mobile site menu, and admin sidebar navigation.</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1990,6 +2353,16 @@
           <t>Assert against `from`, `replyTo`, `subject`, `text`, and `html` directly; do not use a fake preview abstraction.</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2040,6 +2413,16 @@
       <c r="J38" t="inlineStr">
         <is>
           <t>Use `EMAIL_MODE=mock` and `ANTIBOT_MODE=mock`; rerun against a deployed target after shipping the latest worker/site changes.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add logging to cancel bookings
</commit_message>
<xml_diff>
--- a/docs/test-plans/e2e_ui_test_matrix.xlsx
+++ b/docs/test-plans/e2e_ui_test_matrix.xlsx
@@ -185,12 +185,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t/>
+          <t>First command invocation was malformed and did not start the test. Reran the exact T01 Playwright case and it passed cleanly against the deployed mock email/antibot environment.</t>
         </is>
       </c>
     </row>
@@ -247,12 +247,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t/>
+          <t>Headed desktop Chromium run of T04 passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -309,12 +309,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t/>
+          <t>Headed desktop Chromium run of T05 passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -371,12 +371,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t/>
+          <t>Headed desktop Chromium run of T06 passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -433,12 +433,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t/>
+          <t>Initial headed run failed because the test selected a reminder-eligible event on a hidden tab; I fixed the shared evenings helper to reveal the correct tab first. Reran T07 in headed Chromium with yairilluminatetest@gmail.com and it passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -495,12 +495,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t/>
+          <t>Headed desktop Chromium run of T09 passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>booking-flows.spec.ts / mobile-regression.spec.ts</t>
+          <t>mobile-regression.spec.ts :: @mobile contact form valid submit</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -557,12 +557,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t/>
+          <t>Updated the matrix source to the real mobile automation owner. Headed mobile Chromium run passed using the requested customer-email base.</t>
         </is>
       </c>
     </row>
@@ -619,12 +619,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t/>
+          <t>Initial failure was the live confirm endpoint returning "Could not confirm / Internal server error". I deployed a backend fix, then fixed a local E2E navigation-race that was aborting in-flight slot fetches after cancel; the final headed desktop rerun passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -681,12 +681,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t/>
+          <t>Initial headed run expected an inline preview that the current session payment-success page no longer renders. I updated the local E2E assertion to the current success-page contract and the rerun passed.</t>
         </is>
       </c>
     </row>
@@ -733,22 +733,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Needs refactor</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Current automation still contains stale submit-time pay-later assumptions and must be updated to the 2026-03-15 contract.</t>
+          <t>Current shared case matches the 2026-03-15 confirmation-first pay-later contract.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t/>
+          <t>Initial headed run failed because the deployed booking-artifacts test endpoint only accepts @example.test addresses. Reran the pay-later case without the forced Gmail override and it passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -805,12 +805,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t/>
+          <t>Headed desktop Chromium run of the free evening confirmation flow passed cleanly.</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t/>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t/>
+          <t>Headed desktop Chromium run of the paid evening checkout flow passed cleanly.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update turnstile UI test flow
</commit_message>
<xml_diff>
--- a/docs/test-plans/e2e_ui_test_matrix.xlsx
+++ b/docs/test-plans/e2e_ui_test_matrix.xlsx
@@ -1187,10 +1187,10 @@
         <v>Initial run hit live slot contention before reschedule setup completed. I hardened the shared intro-booking helper to recover or restart after slot loss, and the headed rerun passed.</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>Headed mobile Chromium run of the manage-link reschedule flow passed cleanly.</v>
       </c>
     </row>
     <row r="19">
@@ -1533,10 +1533,10 @@
         <v>Content-management coverage.</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>Headed desktop Chromium run of T34 passed cleanly.</v>
       </c>
       <c r="M26" t="str">
         <v/>
@@ -1577,10 +1577,10 @@
         <v>Uses tiny in-memory JPEG payload.</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L27" t="str">
-        <v/>
+        <v>Headed desktop Chromium run of T35 passed cleanly.</v>
       </c>
       <c r="M27" t="str">
         <v/>
@@ -1621,10 +1621,10 @@
         <v>Skips if no editable event exists.</v>
       </c>
       <c r="K28" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L28" t="str">
-        <v/>
+        <v>Headed desktop Chromium run of T36 passed cleanly.</v>
       </c>
       <c r="M28" t="str">
         <v/>
@@ -1709,16 +1709,16 @@
         <v>High-value multi-user regression.</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L30" t="str">
-        <v/>
+        <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the desktop contention case serially in headed Chromium and it passed cleanly.</v>
       </c>
       <c r="M30" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the mobile contention case serially in headed Chromium and it passed cleanly.</v>
       </c>
     </row>
     <row r="31">
@@ -1753,16 +1753,16 @@
         <v>Connects recovery UX with support fallback.</v>
       </c>
       <c r="K31" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L31" t="str">
-        <v/>
+        <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the desktop contention contact fallback case serially in headed Chromium and it passed cleanly.</v>
       </c>
       <c r="M31" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="N31" t="str">
-        <v/>
+        <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the mobile contention contact fallback case serially in headed Chromium and it passed cleanly.</v>
       </c>
     </row>
     <row r="32">
@@ -1797,16 +1797,16 @@
         <v>Core anti-double-booking regression.</v>
       </c>
       <c r="K32" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L32" t="str">
-        <v/>
+        <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the desktop concurrent-race case serially in headed Chromium and it passed cleanly.</v>
       </c>
       <c r="M32" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="N32" t="str">
-        <v/>
+        <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the mobile concurrent-race case serially in headed Chromium and it passed cleanly.</v>
       </c>
     </row>
     <row r="33">
@@ -1841,10 +1841,10 @@
         <v>Form-level antibot behavior with mocked config and fake widget.</v>
       </c>
       <c r="K33" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L33" t="str">
-        <v/>
+        <v>Initial headed run exposed a local mock mismatch: the fake Turnstile booking harness needed a visible slot date, current observability allowlist, and an explicit retry-success route. After those local spec fixes, the rerun passed cleanly.</v>
       </c>
       <c r="M33" t="str">
         <v/>
@@ -1885,10 +1885,10 @@
         <v>Covers anti-bot integration on contact flow.</v>
       </c>
       <c r="K34" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L34" t="str">
-        <v/>
+        <v>Headed desktop Chromium run of the Turnstile contact flow passed cleanly.</v>
       </c>
       <c r="M34" t="str">
         <v/>
@@ -1929,10 +1929,10 @@
         <v>Technical UI guardrail rather than direct product requirement.</v>
       </c>
       <c r="K35" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L35" t="str">
-        <v/>
+        <v>Headed desktop Chromium run of the Turnstile helper scoping check passed cleanly.</v>
       </c>
       <c r="M35" t="str">
         <v/>
@@ -1973,16 +1973,16 @@
         <v>Includes desktop site, mobile site menu, and admin sidebar navigation.</v>
       </c>
       <c r="K36" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="L36" t="str">
-        <v/>
+        <v>Headed desktop Chromium runs of the site desktop nav/footer smoke and admin sidebar smoke both passed cleanly.</v>
       </c>
       <c r="M36" t="str">
-        <v/>
+        <v>PASS</v>
       </c>
       <c r="N36" t="str">
-        <v/>
+        <v>Headed mobile Chromium run of the hamburger navigation smoke passed cleanly.</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
Add Israel coupon booking tests
</commit_message>
<xml_diff>
--- a/docs/test-plans/e2e_ui_test_matrix.xlsx
+++ b/docs/test-plans/e2e_ui_test_matrix.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:R200"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,6 +444,18 @@
       <c r="N1" t="str">
         <v>Mobile Latest Run Comments</v>
       </c>
+      <c r="O1" t="str">
+        <v>Desktop Israel Latest Run Status</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Desktop Israel Latest Run Comments</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Mobile Israel Latest Run Status</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Mobile Israel Latest Run Comments</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -488,6 +500,18 @@
       <c r="N2" t="str">
         <v>Headed mobile Chromium run of @mobile T01 passed cleanly.</v>
       </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -532,6 +556,18 @@
       <c r="N3" t="str">
         <v>Headed mobile Chromium run of @mobile T04 passed cleanly.</v>
       </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -576,6 +612,18 @@
       <c r="N4" t="str">
         <v>Headed mobile Chromium run of @mobile T05 passed cleanly.</v>
       </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -620,6 +668,18 @@
       <c r="N5" t="str">
         <v>Headed mobile Chromium run of @mobile T06 passed cleanly.</v>
       </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -664,6 +724,18 @@
       <c r="N6" t="str">
         <v>Headed mobile Chromium run of @mobile T07 passed cleanly.</v>
       </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -708,6 +780,18 @@
       <c r="N7" t="str">
         <v>Headed mobile Chromium run of @mobile T09 passed cleanly.</v>
       </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -752,6 +836,18 @@
       <c r="N8" t="str">
         <v>Headed mobile Chromium run of @mobile contact form valid submit passed using the requested customer-email base.</v>
       </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -796,6 +892,18 @@
       <c r="N9" t="str">
         <v>Headed mobile Chromium run of the free intro confirm-manage-cancel flow passed cleanly.</v>
       </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -840,6 +948,18 @@
       <c r="N10" t="str">
         <v>Headed mobile Chromium run of the session pay-now checkout recovery flow passed cleanly.</v>
       </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -884,6 +1004,18 @@
       <c r="N11" t="str">
         <v>Headed mobile Chromium run of the pay-later confirmation-first flow passed cleanly.</v>
       </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -928,6 +1060,18 @@
       <c r="N12" t="str">
         <v>Headed mobile Chromium run of the free evening confirmation flow passed cleanly.</v>
       </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -972,6 +1116,18 @@
       <c r="N13" t="str">
         <v>Headed mobile Chromium run of the paid evening checkout flow passed cleanly.</v>
       </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1016,6 +1172,18 @@
       <c r="N14" t="str">
         <v>Headed mobile Chromium run of @mobile T15 passed cleanly.</v>
       </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1060,6 +1228,18 @@
       <c r="N15" t="str">
         <v>Headed mobile Chromium run of @mobile T19 passed cleanly.</v>
       </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1104,6 +1284,18 @@
       <c r="N16" t="str">
         <v>Headed mobile Chromium run of @mobile T20 passed cleanly.</v>
       </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1148,6 +1340,18 @@
       <c r="N17" t="str">
         <v>Headed mobile Chromium run of @mobile T22 passed cleanly.</v>
       </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1192,6 +1396,18 @@
       <c r="N18" t="str">
         <v>Headed mobile Chromium run of the manage-link reschedule flow passed cleanly.</v>
       </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1236,6 +1452,18 @@
       <c r="N19" t="str">
         <v/>
       </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1280,6 +1508,18 @@
       <c r="N20" t="str">
         <v/>
       </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1324,6 +1564,18 @@
       <c r="N21" t="str">
         <v/>
       </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1368,6 +1620,18 @@
       <c r="N22" t="str">
         <v/>
       </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1412,6 +1676,18 @@
       <c r="N23" t="str">
         <v/>
       </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1456,6 +1732,18 @@
       <c r="N24" t="str">
         <v/>
       </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1500,6 +1788,18 @@
       <c r="N25" t="str">
         <v/>
       </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1544,6 +1844,18 @@
       <c r="N26" t="str">
         <v/>
       </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1588,6 +1900,18 @@
       <c r="N27" t="str">
         <v/>
       </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1632,6 +1956,18 @@
       <c r="N28" t="str">
         <v/>
       </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1676,6 +2012,18 @@
       <c r="N29" t="str">
         <v/>
       </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1720,6 +2068,18 @@
       <c r="N30" t="str">
         <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the mobile contention case serially in headed Chromium and it passed cleanly.</v>
       </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1764,6 +2124,18 @@
       <c r="N31" t="str">
         <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the mobile contention contact fallback case serially in headed Chromium and it passed cleanly.</v>
       </c>
+      <c r="O31" t="str">
+        <v/>
+      </c>
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1808,6 +2180,18 @@
       <c r="N32" t="str">
         <v>Parallel desktop/mobile run first collided on shared live intro inventory and produced false failures. Reran the mobile concurrent-race case serially in headed Chromium and it passed cleanly.</v>
       </c>
+      <c r="O32" t="str">
+        <v/>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1852,6 +2236,18 @@
       <c r="N33" t="str">
         <v/>
       </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1896,6 +2292,18 @@
       <c r="N34" t="str">
         <v/>
       </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1940,6 +2348,18 @@
       <c r="N35" t="str">
         <v/>
       </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1984,6 +2404,18 @@
       <c r="N36" t="str">
         <v>Headed mobile Chromium run of the hamburger navigation smoke passed cleanly.</v>
       </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2028,6 +2460,18 @@
       <c r="N37" t="str">
         <v/>
       </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2072,10 +2516,2290 @@
       <c r="N38" t="str">
         <v/>
       </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="O39" t="str">
+        <v/>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="O40" t="str">
+        <v/>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="O41" t="str">
+        <v/>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="O43" t="str">
+        <v/>
+      </c>
+      <c r="P43" t="str">
+        <v/>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="O44" t="str">
+        <v/>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="O46" t="str">
+        <v/>
+      </c>
+      <c r="P46" t="str">
+        <v/>
+      </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="O47" t="str">
+        <v/>
+      </c>
+      <c r="P47" t="str">
+        <v/>
+      </c>
+      <c r="Q47" t="str">
+        <v/>
+      </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="O48" t="str">
+        <v/>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="O49" t="str">
+        <v/>
+      </c>
+      <c r="P49" t="str">
+        <v/>
+      </c>
+      <c r="Q49" t="str">
+        <v/>
+      </c>
+      <c r="R49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="O50" t="str">
+        <v/>
+      </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
+      <c r="R50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="O51" t="str">
+        <v/>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
+      <c r="R51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="O52" t="str">
+        <v/>
+      </c>
+      <c r="P52" t="str">
+        <v/>
+      </c>
+      <c r="Q52" t="str">
+        <v/>
+      </c>
+      <c r="R52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="O53" t="str">
+        <v/>
+      </c>
+      <c r="P53" t="str">
+        <v/>
+      </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
+      <c r="R53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="O54" t="str">
+        <v/>
+      </c>
+      <c r="P54" t="str">
+        <v/>
+      </c>
+      <c r="Q54" t="str">
+        <v/>
+      </c>
+      <c r="R54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="O55" t="str">
+        <v/>
+      </c>
+      <c r="P55" t="str">
+        <v/>
+      </c>
+      <c r="Q55" t="str">
+        <v/>
+      </c>
+      <c r="R55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="O56" t="str">
+        <v/>
+      </c>
+      <c r="P56" t="str">
+        <v/>
+      </c>
+      <c r="Q56" t="str">
+        <v/>
+      </c>
+      <c r="R56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="O57" t="str">
+        <v/>
+      </c>
+      <c r="P57" t="str">
+        <v/>
+      </c>
+      <c r="Q57" t="str">
+        <v/>
+      </c>
+      <c r="R57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="O58" t="str">
+        <v/>
+      </c>
+      <c r="P58" t="str">
+        <v/>
+      </c>
+      <c r="Q58" t="str">
+        <v/>
+      </c>
+      <c r="R58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="O59" t="str">
+        <v/>
+      </c>
+      <c r="P59" t="str">
+        <v/>
+      </c>
+      <c r="Q59" t="str">
+        <v/>
+      </c>
+      <c r="R59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="O60" t="str">
+        <v/>
+      </c>
+      <c r="P60" t="str">
+        <v/>
+      </c>
+      <c r="Q60" t="str">
+        <v/>
+      </c>
+      <c r="R60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="O61" t="str">
+        <v/>
+      </c>
+      <c r="P61" t="str">
+        <v/>
+      </c>
+      <c r="Q61" t="str">
+        <v/>
+      </c>
+      <c r="R61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="O62" t="str">
+        <v/>
+      </c>
+      <c r="P62" t="str">
+        <v/>
+      </c>
+      <c r="Q62" t="str">
+        <v/>
+      </c>
+      <c r="R62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="O63" t="str">
+        <v/>
+      </c>
+      <c r="P63" t="str">
+        <v/>
+      </c>
+      <c r="Q63" t="str">
+        <v/>
+      </c>
+      <c r="R63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="O64" t="str">
+        <v/>
+      </c>
+      <c r="P64" t="str">
+        <v/>
+      </c>
+      <c r="Q64" t="str">
+        <v/>
+      </c>
+      <c r="R64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="O65" t="str">
+        <v/>
+      </c>
+      <c r="P65" t="str">
+        <v/>
+      </c>
+      <c r="Q65" t="str">
+        <v/>
+      </c>
+      <c r="R65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="O66" t="str">
+        <v/>
+      </c>
+      <c r="P66" t="str">
+        <v/>
+      </c>
+      <c r="Q66" t="str">
+        <v/>
+      </c>
+      <c r="R66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="O67" t="str">
+        <v/>
+      </c>
+      <c r="P67" t="str">
+        <v/>
+      </c>
+      <c r="Q67" t="str">
+        <v/>
+      </c>
+      <c r="R67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="O68" t="str">
+        <v/>
+      </c>
+      <c r="P68" t="str">
+        <v/>
+      </c>
+      <c r="Q68" t="str">
+        <v/>
+      </c>
+      <c r="R68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="O69" t="str">
+        <v/>
+      </c>
+      <c r="P69" t="str">
+        <v/>
+      </c>
+      <c r="Q69" t="str">
+        <v/>
+      </c>
+      <c r="R69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="O70" t="str">
+        <v/>
+      </c>
+      <c r="P70" t="str">
+        <v/>
+      </c>
+      <c r="Q70" t="str">
+        <v/>
+      </c>
+      <c r="R70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="O71" t="str">
+        <v/>
+      </c>
+      <c r="P71" t="str">
+        <v/>
+      </c>
+      <c r="Q71" t="str">
+        <v/>
+      </c>
+      <c r="R71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="O72" t="str">
+        <v/>
+      </c>
+      <c r="P72" t="str">
+        <v/>
+      </c>
+      <c r="Q72" t="str">
+        <v/>
+      </c>
+      <c r="R72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="O73" t="str">
+        <v/>
+      </c>
+      <c r="P73" t="str">
+        <v/>
+      </c>
+      <c r="Q73" t="str">
+        <v/>
+      </c>
+      <c r="R73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="O74" t="str">
+        <v/>
+      </c>
+      <c r="P74" t="str">
+        <v/>
+      </c>
+      <c r="Q74" t="str">
+        <v/>
+      </c>
+      <c r="R74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="O75" t="str">
+        <v/>
+      </c>
+      <c r="P75" t="str">
+        <v/>
+      </c>
+      <c r="Q75" t="str">
+        <v/>
+      </c>
+      <c r="R75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="O76" t="str">
+        <v/>
+      </c>
+      <c r="P76" t="str">
+        <v/>
+      </c>
+      <c r="Q76" t="str">
+        <v/>
+      </c>
+      <c r="R76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="O77" t="str">
+        <v/>
+      </c>
+      <c r="P77" t="str">
+        <v/>
+      </c>
+      <c r="Q77" t="str">
+        <v/>
+      </c>
+      <c r="R77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="O78" t="str">
+        <v/>
+      </c>
+      <c r="P78" t="str">
+        <v/>
+      </c>
+      <c r="Q78" t="str">
+        <v/>
+      </c>
+      <c r="R78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="O79" t="str">
+        <v/>
+      </c>
+      <c r="P79" t="str">
+        <v/>
+      </c>
+      <c r="Q79" t="str">
+        <v/>
+      </c>
+      <c r="R79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="O80" t="str">
+        <v/>
+      </c>
+      <c r="P80" t="str">
+        <v/>
+      </c>
+      <c r="Q80" t="str">
+        <v/>
+      </c>
+      <c r="R80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="O81" t="str">
+        <v/>
+      </c>
+      <c r="P81" t="str">
+        <v/>
+      </c>
+      <c r="Q81" t="str">
+        <v/>
+      </c>
+      <c r="R81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="O82" t="str">
+        <v/>
+      </c>
+      <c r="P82" t="str">
+        <v/>
+      </c>
+      <c r="Q82" t="str">
+        <v/>
+      </c>
+      <c r="R82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="O83" t="str">
+        <v/>
+      </c>
+      <c r="P83" t="str">
+        <v/>
+      </c>
+      <c r="Q83" t="str">
+        <v/>
+      </c>
+      <c r="R83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="O84" t="str">
+        <v/>
+      </c>
+      <c r="P84" t="str">
+        <v/>
+      </c>
+      <c r="Q84" t="str">
+        <v/>
+      </c>
+      <c r="R84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="O85" t="str">
+        <v/>
+      </c>
+      <c r="P85" t="str">
+        <v/>
+      </c>
+      <c r="Q85" t="str">
+        <v/>
+      </c>
+      <c r="R85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="O86" t="str">
+        <v/>
+      </c>
+      <c r="P86" t="str">
+        <v/>
+      </c>
+      <c r="Q86" t="str">
+        <v/>
+      </c>
+      <c r="R86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="O87" t="str">
+        <v/>
+      </c>
+      <c r="P87" t="str">
+        <v/>
+      </c>
+      <c r="Q87" t="str">
+        <v/>
+      </c>
+      <c r="R87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="O88" t="str">
+        <v/>
+      </c>
+      <c r="P88" t="str">
+        <v/>
+      </c>
+      <c r="Q88" t="str">
+        <v/>
+      </c>
+      <c r="R88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="O89" t="str">
+        <v/>
+      </c>
+      <c r="P89" t="str">
+        <v/>
+      </c>
+      <c r="Q89" t="str">
+        <v/>
+      </c>
+      <c r="R89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="O90" t="str">
+        <v/>
+      </c>
+      <c r="P90" t="str">
+        <v/>
+      </c>
+      <c r="Q90" t="str">
+        <v/>
+      </c>
+      <c r="R90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="O91" t="str">
+        <v/>
+      </c>
+      <c r="P91" t="str">
+        <v/>
+      </c>
+      <c r="Q91" t="str">
+        <v/>
+      </c>
+      <c r="R91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="O92" t="str">
+        <v/>
+      </c>
+      <c r="P92" t="str">
+        <v/>
+      </c>
+      <c r="Q92" t="str">
+        <v/>
+      </c>
+      <c r="R92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="O93" t="str">
+        <v/>
+      </c>
+      <c r="P93" t="str">
+        <v/>
+      </c>
+      <c r="Q93" t="str">
+        <v/>
+      </c>
+      <c r="R93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="O94" t="str">
+        <v/>
+      </c>
+      <c r="P94" t="str">
+        <v/>
+      </c>
+      <c r="Q94" t="str">
+        <v/>
+      </c>
+      <c r="R94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="O95" t="str">
+        <v/>
+      </c>
+      <c r="P95" t="str">
+        <v/>
+      </c>
+      <c r="Q95" t="str">
+        <v/>
+      </c>
+      <c r="R95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="O96" t="str">
+        <v/>
+      </c>
+      <c r="P96" t="str">
+        <v/>
+      </c>
+      <c r="Q96" t="str">
+        <v/>
+      </c>
+      <c r="R96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="O97" t="str">
+        <v/>
+      </c>
+      <c r="P97" t="str">
+        <v/>
+      </c>
+      <c r="Q97" t="str">
+        <v/>
+      </c>
+      <c r="R97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="O98" t="str">
+        <v/>
+      </c>
+      <c r="P98" t="str">
+        <v/>
+      </c>
+      <c r="Q98" t="str">
+        <v/>
+      </c>
+      <c r="R98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="O99" t="str">
+        <v/>
+      </c>
+      <c r="P99" t="str">
+        <v/>
+      </c>
+      <c r="Q99" t="str">
+        <v/>
+      </c>
+      <c r="R99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="O100" t="str">
+        <v/>
+      </c>
+      <c r="P100" t="str">
+        <v/>
+      </c>
+      <c r="Q100" t="str">
+        <v/>
+      </c>
+      <c r="R100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="O101" t="str">
+        <v/>
+      </c>
+      <c r="P101" t="str">
+        <v/>
+      </c>
+      <c r="Q101" t="str">
+        <v/>
+      </c>
+      <c r="R101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="O102" t="str">
+        <v/>
+      </c>
+      <c r="P102" t="str">
+        <v/>
+      </c>
+      <c r="Q102" t="str">
+        <v/>
+      </c>
+      <c r="R102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="O103" t="str">
+        <v/>
+      </c>
+      <c r="P103" t="str">
+        <v/>
+      </c>
+      <c r="Q103" t="str">
+        <v/>
+      </c>
+      <c r="R103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="O104" t="str">
+        <v/>
+      </c>
+      <c r="P104" t="str">
+        <v/>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
+      </c>
+      <c r="R104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v/>
+      </c>
+      <c r="Q105" t="str">
+        <v/>
+      </c>
+      <c r="R105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="O106" t="str">
+        <v/>
+      </c>
+      <c r="P106" t="str">
+        <v/>
+      </c>
+      <c r="Q106" t="str">
+        <v/>
+      </c>
+      <c r="R106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="O107" t="str">
+        <v/>
+      </c>
+      <c r="P107" t="str">
+        <v/>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="O108" t="str">
+        <v/>
+      </c>
+      <c r="P108" t="str">
+        <v/>
+      </c>
+      <c r="Q108" t="str">
+        <v/>
+      </c>
+      <c r="R108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="O109" t="str">
+        <v/>
+      </c>
+      <c r="P109" t="str">
+        <v/>
+      </c>
+      <c r="Q109" t="str">
+        <v/>
+      </c>
+      <c r="R109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="O110" t="str">
+        <v/>
+      </c>
+      <c r="P110" t="str">
+        <v/>
+      </c>
+      <c r="Q110" t="str">
+        <v/>
+      </c>
+      <c r="R110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="O112" t="str">
+        <v/>
+      </c>
+      <c r="P112" t="str">
+        <v/>
+      </c>
+      <c r="Q112" t="str">
+        <v/>
+      </c>
+      <c r="R112" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="O113" t="str">
+        <v/>
+      </c>
+      <c r="P113" t="str">
+        <v/>
+      </c>
+      <c r="Q113" t="str">
+        <v/>
+      </c>
+      <c r="R113" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="O114" t="str">
+        <v/>
+      </c>
+      <c r="P114" t="str">
+        <v/>
+      </c>
+      <c r="Q114" t="str">
+        <v/>
+      </c>
+      <c r="R114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="O115" t="str">
+        <v/>
+      </c>
+      <c r="P115" t="str">
+        <v/>
+      </c>
+      <c r="Q115" t="str">
+        <v/>
+      </c>
+      <c r="R115" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="O116" t="str">
+        <v/>
+      </c>
+      <c r="P116" t="str">
+        <v/>
+      </c>
+      <c r="Q116" t="str">
+        <v/>
+      </c>
+      <c r="R116" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="O117" t="str">
+        <v/>
+      </c>
+      <c r="P117" t="str">
+        <v/>
+      </c>
+      <c r="Q117" t="str">
+        <v/>
+      </c>
+      <c r="R117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="O118" t="str">
+        <v/>
+      </c>
+      <c r="P118" t="str">
+        <v/>
+      </c>
+      <c r="Q118" t="str">
+        <v/>
+      </c>
+      <c r="R118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="O119" t="str">
+        <v/>
+      </c>
+      <c r="P119" t="str">
+        <v/>
+      </c>
+      <c r="Q119" t="str">
+        <v/>
+      </c>
+      <c r="R119" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="O120" t="str">
+        <v/>
+      </c>
+      <c r="P120" t="str">
+        <v/>
+      </c>
+      <c r="Q120" t="str">
+        <v/>
+      </c>
+      <c r="R120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="O121" t="str">
+        <v/>
+      </c>
+      <c r="P121" t="str">
+        <v/>
+      </c>
+      <c r="Q121" t="str">
+        <v/>
+      </c>
+      <c r="R121" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="O122" t="str">
+        <v/>
+      </c>
+      <c r="P122" t="str">
+        <v/>
+      </c>
+      <c r="Q122" t="str">
+        <v/>
+      </c>
+      <c r="R122" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="O123" t="str">
+        <v/>
+      </c>
+      <c r="P123" t="str">
+        <v/>
+      </c>
+      <c r="Q123" t="str">
+        <v/>
+      </c>
+      <c r="R123" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="O124" t="str">
+        <v/>
+      </c>
+      <c r="P124" t="str">
+        <v/>
+      </c>
+      <c r="Q124" t="str">
+        <v/>
+      </c>
+      <c r="R124" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="O125" t="str">
+        <v/>
+      </c>
+      <c r="P125" t="str">
+        <v/>
+      </c>
+      <c r="Q125" t="str">
+        <v/>
+      </c>
+      <c r="R125" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="O126" t="str">
+        <v/>
+      </c>
+      <c r="P126" t="str">
+        <v/>
+      </c>
+      <c r="Q126" t="str">
+        <v/>
+      </c>
+      <c r="R126" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="O127" t="str">
+        <v/>
+      </c>
+      <c r="P127" t="str">
+        <v/>
+      </c>
+      <c r="Q127" t="str">
+        <v/>
+      </c>
+      <c r="R127" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="O128" t="str">
+        <v/>
+      </c>
+      <c r="P128" t="str">
+        <v/>
+      </c>
+      <c r="Q128" t="str">
+        <v/>
+      </c>
+      <c r="R128" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="O129" t="str">
+        <v/>
+      </c>
+      <c r="P129" t="str">
+        <v/>
+      </c>
+      <c r="Q129" t="str">
+        <v/>
+      </c>
+      <c r="R129" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="O130" t="str">
+        <v/>
+      </c>
+      <c r="P130" t="str">
+        <v/>
+      </c>
+      <c r="Q130" t="str">
+        <v/>
+      </c>
+      <c r="R130" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="O131" t="str">
+        <v/>
+      </c>
+      <c r="P131" t="str">
+        <v/>
+      </c>
+      <c r="Q131" t="str">
+        <v/>
+      </c>
+      <c r="R131" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="O132" t="str">
+        <v/>
+      </c>
+      <c r="P132" t="str">
+        <v/>
+      </c>
+      <c r="Q132" t="str">
+        <v/>
+      </c>
+      <c r="R132" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="O133" t="str">
+        <v/>
+      </c>
+      <c r="P133" t="str">
+        <v/>
+      </c>
+      <c r="Q133" t="str">
+        <v/>
+      </c>
+      <c r="R133" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="O134" t="str">
+        <v/>
+      </c>
+      <c r="P134" t="str">
+        <v/>
+      </c>
+      <c r="Q134" t="str">
+        <v/>
+      </c>
+      <c r="R134" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="O135" t="str">
+        <v/>
+      </c>
+      <c r="P135" t="str">
+        <v/>
+      </c>
+      <c r="Q135" t="str">
+        <v/>
+      </c>
+      <c r="R135" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="O136" t="str">
+        <v/>
+      </c>
+      <c r="P136" t="str">
+        <v/>
+      </c>
+      <c r="Q136" t="str">
+        <v/>
+      </c>
+      <c r="R136" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="O137" t="str">
+        <v/>
+      </c>
+      <c r="P137" t="str">
+        <v/>
+      </c>
+      <c r="Q137" t="str">
+        <v/>
+      </c>
+      <c r="R137" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="O138" t="str">
+        <v/>
+      </c>
+      <c r="P138" t="str">
+        <v/>
+      </c>
+      <c r="Q138" t="str">
+        <v/>
+      </c>
+      <c r="R138" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="O139" t="str">
+        <v/>
+      </c>
+      <c r="P139" t="str">
+        <v/>
+      </c>
+      <c r="Q139" t="str">
+        <v/>
+      </c>
+      <c r="R139" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="O140" t="str">
+        <v/>
+      </c>
+      <c r="P140" t="str">
+        <v/>
+      </c>
+      <c r="Q140" t="str">
+        <v/>
+      </c>
+      <c r="R140" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="O141" t="str">
+        <v/>
+      </c>
+      <c r="P141" t="str">
+        <v/>
+      </c>
+      <c r="Q141" t="str">
+        <v/>
+      </c>
+      <c r="R141" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="O142" t="str">
+        <v/>
+      </c>
+      <c r="P142" t="str">
+        <v/>
+      </c>
+      <c r="Q142" t="str">
+        <v/>
+      </c>
+      <c r="R142" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="O143" t="str">
+        <v/>
+      </c>
+      <c r="P143" t="str">
+        <v/>
+      </c>
+      <c r="Q143" t="str">
+        <v/>
+      </c>
+      <c r="R143" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="O144" t="str">
+        <v/>
+      </c>
+      <c r="P144" t="str">
+        <v/>
+      </c>
+      <c r="Q144" t="str">
+        <v/>
+      </c>
+      <c r="R144" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="O145" t="str">
+        <v/>
+      </c>
+      <c r="P145" t="str">
+        <v/>
+      </c>
+      <c r="Q145" t="str">
+        <v/>
+      </c>
+      <c r="R145" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="O146" t="str">
+        <v/>
+      </c>
+      <c r="P146" t="str">
+        <v/>
+      </c>
+      <c r="Q146" t="str">
+        <v/>
+      </c>
+      <c r="R146" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="O147" t="str">
+        <v/>
+      </c>
+      <c r="P147" t="str">
+        <v/>
+      </c>
+      <c r="Q147" t="str">
+        <v/>
+      </c>
+      <c r="R147" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="O148" t="str">
+        <v/>
+      </c>
+      <c r="P148" t="str">
+        <v/>
+      </c>
+      <c r="Q148" t="str">
+        <v/>
+      </c>
+      <c r="R148" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="O149" t="str">
+        <v/>
+      </c>
+      <c r="P149" t="str">
+        <v/>
+      </c>
+      <c r="Q149" t="str">
+        <v/>
+      </c>
+      <c r="R149" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="O150" t="str">
+        <v/>
+      </c>
+      <c r="P150" t="str">
+        <v/>
+      </c>
+      <c r="Q150" t="str">
+        <v/>
+      </c>
+      <c r="R150" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="O151" t="str">
+        <v/>
+      </c>
+      <c r="P151" t="str">
+        <v/>
+      </c>
+      <c r="Q151" t="str">
+        <v/>
+      </c>
+      <c r="R151" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="O152" t="str">
+        <v/>
+      </c>
+      <c r="P152" t="str">
+        <v/>
+      </c>
+      <c r="Q152" t="str">
+        <v/>
+      </c>
+      <c r="R152" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="O153" t="str">
+        <v/>
+      </c>
+      <c r="P153" t="str">
+        <v/>
+      </c>
+      <c r="Q153" t="str">
+        <v/>
+      </c>
+      <c r="R153" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="O154" t="str">
+        <v/>
+      </c>
+      <c r="P154" t="str">
+        <v/>
+      </c>
+      <c r="Q154" t="str">
+        <v/>
+      </c>
+      <c r="R154" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="O155" t="str">
+        <v/>
+      </c>
+      <c r="P155" t="str">
+        <v/>
+      </c>
+      <c r="Q155" t="str">
+        <v/>
+      </c>
+      <c r="R155" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="O156" t="str">
+        <v/>
+      </c>
+      <c r="P156" t="str">
+        <v/>
+      </c>
+      <c r="Q156" t="str">
+        <v/>
+      </c>
+      <c r="R156" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="O157" t="str">
+        <v/>
+      </c>
+      <c r="P157" t="str">
+        <v/>
+      </c>
+      <c r="Q157" t="str">
+        <v/>
+      </c>
+      <c r="R157" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="O158" t="str">
+        <v/>
+      </c>
+      <c r="P158" t="str">
+        <v/>
+      </c>
+      <c r="Q158" t="str">
+        <v/>
+      </c>
+      <c r="R158" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="O159" t="str">
+        <v/>
+      </c>
+      <c r="P159" t="str">
+        <v/>
+      </c>
+      <c r="Q159" t="str">
+        <v/>
+      </c>
+      <c r="R159" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="O160" t="str">
+        <v/>
+      </c>
+      <c r="P160" t="str">
+        <v/>
+      </c>
+      <c r="Q160" t="str">
+        <v/>
+      </c>
+      <c r="R160" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="O161" t="str">
+        <v/>
+      </c>
+      <c r="P161" t="str">
+        <v/>
+      </c>
+      <c r="Q161" t="str">
+        <v/>
+      </c>
+      <c r="R161" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="O162" t="str">
+        <v/>
+      </c>
+      <c r="P162" t="str">
+        <v/>
+      </c>
+      <c r="Q162" t="str">
+        <v/>
+      </c>
+      <c r="R162" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="O163" t="str">
+        <v/>
+      </c>
+      <c r="P163" t="str">
+        <v/>
+      </c>
+      <c r="Q163" t="str">
+        <v/>
+      </c>
+      <c r="R163" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="O164" t="str">
+        <v/>
+      </c>
+      <c r="P164" t="str">
+        <v/>
+      </c>
+      <c r="Q164" t="str">
+        <v/>
+      </c>
+      <c r="R164" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="O165" t="str">
+        <v/>
+      </c>
+      <c r="P165" t="str">
+        <v/>
+      </c>
+      <c r="Q165" t="str">
+        <v/>
+      </c>
+      <c r="R165" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="O166" t="str">
+        <v/>
+      </c>
+      <c r="P166" t="str">
+        <v/>
+      </c>
+      <c r="Q166" t="str">
+        <v/>
+      </c>
+      <c r="R166" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="O167" t="str">
+        <v/>
+      </c>
+      <c r="P167" t="str">
+        <v/>
+      </c>
+      <c r="Q167" t="str">
+        <v/>
+      </c>
+      <c r="R167" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="O168" t="str">
+        <v/>
+      </c>
+      <c r="P168" t="str">
+        <v/>
+      </c>
+      <c r="Q168" t="str">
+        <v/>
+      </c>
+      <c r="R168" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="O169" t="str">
+        <v/>
+      </c>
+      <c r="P169" t="str">
+        <v/>
+      </c>
+      <c r="Q169" t="str">
+        <v/>
+      </c>
+      <c r="R169" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="O170" t="str">
+        <v/>
+      </c>
+      <c r="P170" t="str">
+        <v/>
+      </c>
+      <c r="Q170" t="str">
+        <v/>
+      </c>
+      <c r="R170" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="O171" t="str">
+        <v/>
+      </c>
+      <c r="P171" t="str">
+        <v/>
+      </c>
+      <c r="Q171" t="str">
+        <v/>
+      </c>
+      <c r="R171" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="O172" t="str">
+        <v/>
+      </c>
+      <c r="P172" t="str">
+        <v/>
+      </c>
+      <c r="Q172" t="str">
+        <v/>
+      </c>
+      <c r="R172" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="O173" t="str">
+        <v/>
+      </c>
+      <c r="P173" t="str">
+        <v/>
+      </c>
+      <c r="Q173" t="str">
+        <v/>
+      </c>
+      <c r="R173" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="O174" t="str">
+        <v/>
+      </c>
+      <c r="P174" t="str">
+        <v/>
+      </c>
+      <c r="Q174" t="str">
+        <v/>
+      </c>
+      <c r="R174" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="O175" t="str">
+        <v/>
+      </c>
+      <c r="P175" t="str">
+        <v/>
+      </c>
+      <c r="Q175" t="str">
+        <v/>
+      </c>
+      <c r="R175" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="O176" t="str">
+        <v/>
+      </c>
+      <c r="P176" t="str">
+        <v/>
+      </c>
+      <c r="Q176" t="str">
+        <v/>
+      </c>
+      <c r="R176" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="O177" t="str">
+        <v/>
+      </c>
+      <c r="P177" t="str">
+        <v/>
+      </c>
+      <c r="Q177" t="str">
+        <v/>
+      </c>
+      <c r="R177" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="O178" t="str">
+        <v/>
+      </c>
+      <c r="P178" t="str">
+        <v/>
+      </c>
+      <c r="Q178" t="str">
+        <v/>
+      </c>
+      <c r="R178" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="O179" t="str">
+        <v/>
+      </c>
+      <c r="P179" t="str">
+        <v/>
+      </c>
+      <c r="Q179" t="str">
+        <v/>
+      </c>
+      <c r="R179" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="O180" t="str">
+        <v/>
+      </c>
+      <c r="P180" t="str">
+        <v/>
+      </c>
+      <c r="Q180" t="str">
+        <v/>
+      </c>
+      <c r="R180" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="O181" t="str">
+        <v/>
+      </c>
+      <c r="P181" t="str">
+        <v/>
+      </c>
+      <c r="Q181" t="str">
+        <v/>
+      </c>
+      <c r="R181" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="O182" t="str">
+        <v/>
+      </c>
+      <c r="P182" t="str">
+        <v/>
+      </c>
+      <c r="Q182" t="str">
+        <v/>
+      </c>
+      <c r="R182" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="O183" t="str">
+        <v/>
+      </c>
+      <c r="P183" t="str">
+        <v/>
+      </c>
+      <c r="Q183" t="str">
+        <v/>
+      </c>
+      <c r="R183" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="O184" t="str">
+        <v/>
+      </c>
+      <c r="P184" t="str">
+        <v/>
+      </c>
+      <c r="Q184" t="str">
+        <v/>
+      </c>
+      <c r="R184" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="O185" t="str">
+        <v/>
+      </c>
+      <c r="P185" t="str">
+        <v/>
+      </c>
+      <c r="Q185" t="str">
+        <v/>
+      </c>
+      <c r="R185" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="O186" t="str">
+        <v/>
+      </c>
+      <c r="P186" t="str">
+        <v/>
+      </c>
+      <c r="Q186" t="str">
+        <v/>
+      </c>
+      <c r="R186" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="O187" t="str">
+        <v/>
+      </c>
+      <c r="P187" t="str">
+        <v/>
+      </c>
+      <c r="Q187" t="str">
+        <v/>
+      </c>
+      <c r="R187" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="O188" t="str">
+        <v/>
+      </c>
+      <c r="P188" t="str">
+        <v/>
+      </c>
+      <c r="Q188" t="str">
+        <v/>
+      </c>
+      <c r="R188" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="O189" t="str">
+        <v/>
+      </c>
+      <c r="P189" t="str">
+        <v/>
+      </c>
+      <c r="Q189" t="str">
+        <v/>
+      </c>
+      <c r="R189" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="O190" t="str">
+        <v/>
+      </c>
+      <c r="P190" t="str">
+        <v/>
+      </c>
+      <c r="Q190" t="str">
+        <v/>
+      </c>
+      <c r="R190" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="O191" t="str">
+        <v/>
+      </c>
+      <c r="P191" t="str">
+        <v/>
+      </c>
+      <c r="Q191" t="str">
+        <v/>
+      </c>
+      <c r="R191" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="O192" t="str">
+        <v/>
+      </c>
+      <c r="P192" t="str">
+        <v/>
+      </c>
+      <c r="Q192" t="str">
+        <v/>
+      </c>
+      <c r="R192" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="O193" t="str">
+        <v/>
+      </c>
+      <c r="P193" t="str">
+        <v/>
+      </c>
+      <c r="Q193" t="str">
+        <v/>
+      </c>
+      <c r="R193" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="O194" t="str">
+        <v/>
+      </c>
+      <c r="P194" t="str">
+        <v/>
+      </c>
+      <c r="Q194" t="str">
+        <v/>
+      </c>
+      <c r="R194" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="O195" t="str">
+        <v/>
+      </c>
+      <c r="P195" t="str">
+        <v/>
+      </c>
+      <c r="Q195" t="str">
+        <v/>
+      </c>
+      <c r="R195" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="O196" t="str">
+        <v/>
+      </c>
+      <c r="P196" t="str">
+        <v/>
+      </c>
+      <c r="Q196" t="str">
+        <v/>
+      </c>
+      <c r="R196" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="O197" t="str">
+        <v/>
+      </c>
+      <c r="P197" t="str">
+        <v/>
+      </c>
+      <c r="Q197" t="str">
+        <v/>
+      </c>
+      <c r="R197" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="O198" t="str">
+        <v/>
+      </c>
+      <c r="P198" t="str">
+        <v/>
+      </c>
+      <c r="Q198" t="str">
+        <v/>
+      </c>
+      <c r="R198" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="O199" t="str">
+        <v/>
+      </c>
+      <c r="P199" t="str">
+        <v/>
+      </c>
+      <c r="Q199" t="str">
+        <v/>
+      </c>
+      <c r="R199" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="O200" t="str">
+        <v/>
+      </c>
+      <c r="P200" t="str">
+        <v/>
+      </c>
+      <c r="Q200" t="str">
+        <v/>
+      </c>
+      <c r="R200" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R200"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update delete prefix cleanup
</commit_message>
<xml_diff>
--- a/docs/test-plans/e2e_ui_test_matrix.xlsx
+++ b/docs/test-plans/e2e_ui_test_matrix.xlsx
@@ -398,7 +398,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:R200"/>
   <sheetData>
     <row r="1">
@@ -500,17 +500,25 @@
       <c r="N2" t="str">
         <v>Headed mobile Chromium run of @mobile T01 passed cleanly.</v>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Israel banner appeared on home and sessions, stayed sticky on the home scroll path, and did not appear on evenings. Sessions required scrolling #session-types into view.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Israel banner appeared on home and sessions in headed mobile Chromium, and evenings intentionally showed no coupon banner.</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -948,17 +956,25 @@
       <c r="N10" t="str">
         <v>Headed mobile Chromium run of the session pay-now checkout recovery flow passed cleanly.</v>
       </c>
-      <c r="O10" t="str">
-        <v/>
-      </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-      <c r="Q10" t="str">
-        <v/>
-      </c>
-      <c r="R10" t="str">
-        <v/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Both discounted pay-now session variants passed: banner-applied and remove-then-manual-review apply. DB, payment, and admin all showed the discounted amount with coupon code ISRAEL.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Both discounted mobile pay-now session variants passed after fixing origin-scoped coupon clearing and slot-contention retry. DB, payment, and admin all showed the discounted amount with coupon code ISRAEL.</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1004,17 +1020,25 @@
       <c r="N11" t="str">
         <v>Headed mobile Chromium run of the pay-later confirmation-first flow passed cleanly.</v>
       </c>
-      <c r="O11" t="str">
-        <v/>
-      </c>
-      <c r="P11" t="str">
-        <v/>
-      </c>
-      <c r="Q11" t="str">
-        <v/>
-      </c>
-      <c r="R11" t="str">
-        <v/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Both discounted pay-later session variants passed: banner-applied and remove-then-manual-review apply. After confirmation, DB, pending payment, and admin all showed the discounted amount with coupon code ISRAEL.</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Both discounted mobile pay-later session variants passed. After confirmation, DB, pending payment, and admin all showed the discounted amount with coupon code ISRAEL.</t>
+        </is>
       </c>
     </row>
     <row r="12">

</xml_diff>